<commit_message>
feat: metas por pasta da planilha Totais
As metas da pasta e do total passam a vir de "(BASE) - Metas Polybalas -
Totais" (META e CARTEIRA, linha PLB = total), no lugar da planilha antiga
por vendedor. Entra "(BASE) - Metas Polybalas - Fornecedores" como
referência opcional, e produtos foco passa a ser "(BASE) - Produtos Focos
KPI's". O total conta todas as vendas do arquivo; pasta sem fornecedor
(como TLV) fica fora das telas, com aviso. Aceita "R$ 650.000,00".
</commit_message>
<xml_diff>
--- a/tools/exemplos/(BASE) - Metas Polybalas - KPI's e Produtos Focos.xlsx
+++ b/tools/exemplos/(BASE) - Metas Polybalas - KPI's e Produtos Focos.xlsx
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G2" t="n">
-        <v>6358.21</v>
+        <v>4277.94</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>33</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -545,10 +545,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="G4" t="n">
-        <v>12558.91</v>
+        <v>13072.96</v>
       </c>
     </row>
     <row r="5">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6">
@@ -604,10 +604,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G6" t="n">
-        <v>18054.38</v>
+        <v>18012.31</v>
       </c>
     </row>
     <row r="7">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8">
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G8" t="n">
-        <v>5631.47</v>
+        <v>3010.14</v>
       </c>
     </row>
     <row r="9">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
@@ -722,10 +722,10 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G10" t="n">
-        <v>9764.360000000001</v>
+        <v>8297.92</v>
       </c>
     </row>
     <row r="11">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12">
@@ -781,10 +781,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G12" t="n">
-        <v>19345.29</v>
+        <v>9137.870000000001</v>
       </c>
     </row>
     <row r="13">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14">
@@ -840,10 +840,10 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G14" t="n">
-        <v>6804</v>
+        <v>3840.9</v>
       </c>
     </row>
     <row r="15">
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
@@ -899,10 +899,10 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G16" t="n">
-        <v>8749.5</v>
+        <v>13839.3</v>
       </c>
     </row>
     <row r="17">
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18">
@@ -958,10 +958,10 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G18" t="n">
-        <v>13309.31</v>
+        <v>20995.87</v>
       </c>
     </row>
     <row r="19">
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20">
@@ -1017,10 +1017,10 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="G20" t="n">
-        <v>6588.09</v>
+        <v>5892.45</v>
       </c>
     </row>
     <row r="21">
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22">
@@ -1076,10 +1076,10 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G22" t="n">
-        <v>7266.35</v>
+        <v>8300.82</v>
       </c>
     </row>
     <row r="23">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
     </row>
     <row r="24">
@@ -1135,10 +1135,10 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G24" t="n">
-        <v>14818.28</v>
+        <v>9296.870000000001</v>
       </c>
     </row>
     <row r="25">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26">
@@ -1197,7 +1197,7 @@
         <v>31</v>
       </c>
       <c r="G26" t="n">
-        <v>6255.02</v>
+        <v>4844.29</v>
       </c>
     </row>
     <row r="27">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28">
@@ -1253,10 +1253,10 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G28" t="n">
-        <v>12362.93</v>
+        <v>13127.75</v>
       </c>
     </row>
     <row r="29">
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G30" t="n">
-        <v>12588.43</v>
+        <v>14105.32</v>
       </c>
     </row>
     <row r="31">
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
     </row>
     <row r="32">
@@ -1371,10 +1371,10 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G32" t="n">
-        <v>5858.87</v>
+        <v>6667.02</v>
       </c>
     </row>
     <row r="33">
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34">
@@ -1430,10 +1430,10 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="G34" t="n">
-        <v>10267.32</v>
+        <v>10512</v>
       </c>
     </row>
     <row r="35">
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36">
@@ -1489,10 +1489,10 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="G36" t="n">
-        <v>20466.51</v>
+        <v>15215.85</v>
       </c>
     </row>
     <row r="37">
@@ -1520,7 +1520,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>92</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38">
@@ -1548,10 +1548,10 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="G38" t="n">
-        <v>6248.19</v>
+        <v>6063.31</v>
       </c>
     </row>
     <row r="39">
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="40">
@@ -1610,7 +1610,7 @@
         <v>60</v>
       </c>
       <c r="G40" t="n">
-        <v>6839.37</v>
+        <v>13094.6</v>
       </c>
     </row>
     <row r="41">
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42">
@@ -1666,10 +1666,10 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G42" t="n">
-        <v>13003.32</v>
+        <v>14640.48</v>
       </c>
     </row>
     <row r="43">
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
     </row>
     <row r="44">
@@ -1725,10 +1725,10 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G44" t="n">
-        <v>3166.35</v>
+        <v>6398.52</v>
       </c>
     </row>
     <row r="45">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46">
@@ -1784,10 +1784,10 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="G46" t="n">
-        <v>13191.3</v>
+        <v>11394.43</v>
       </c>
     </row>
     <row r="47">
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="48">
@@ -1843,10 +1843,10 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G48" t="n">
-        <v>13286.68</v>
+        <v>17037.05</v>
       </c>
     </row>
     <row r="49">
@@ -1874,7 +1874,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="50">
@@ -1902,10 +1902,10 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G50" t="n">
-        <v>6904.47</v>
+        <v>5793.29</v>
       </c>
     </row>
     <row r="51">
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
     </row>
     <row r="52">
@@ -1961,10 +1961,10 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G52" t="n">
-        <v>13513.74</v>
+        <v>7620.25</v>
       </c>
     </row>
     <row r="53">
@@ -1992,7 +1992,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54">
@@ -2020,10 +2020,10 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="G54" t="n">
-        <v>17663.76</v>
+        <v>9397.309999999999</v>
       </c>
     </row>
     <row r="55">
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="56">
@@ -2079,10 +2079,10 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G56" t="n">
-        <v>4258.69</v>
+        <v>6707.83</v>
       </c>
     </row>
     <row r="57">
@@ -2110,7 +2110,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="58">
@@ -2138,10 +2138,10 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G58" t="n">
-        <v>6227.34</v>
+        <v>8080.88</v>
       </c>
     </row>
     <row r="59">
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>59</v>
+        <v>71</v>
       </c>
     </row>
     <row r="60">
@@ -2197,10 +2197,10 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G60" t="n">
-        <v>17012.43</v>
+        <v>15135.2</v>
       </c>
     </row>
     <row r="61">
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Televendas (TLV) como pasta nos painéis
Venda de vendedor "P-TLV-" ou do supervisor Televendas conta na TLV e no
total, não na pasta do fornecedor, para as pastas somarem o total da
planilha Totais. Os nomes só servem para essa marcação e não são guardados.
</commit_message>
<xml_diff>
--- a/tools/exemplos/(BASE) - Metas Polybalas - KPI's e Produtos Focos.xlsx
+++ b/tools/exemplos/(BASE) - Metas Polybalas - KPI's e Produtos Focos.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2231,6 +2231,360 @@
         <v>95</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>FOCO PILHAS</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>33</v>
+      </c>
+      <c r="G62" t="n">
+        <v>5231.35</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>FOCO SANDÁLIAS</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>61</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>FOCO HIGIENE</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>53</v>
+      </c>
+      <c r="G64" t="n">
+        <v>8533.26</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>FOCO ESPONJAS</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>61</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>FOCO CABELOS</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>82</v>
+      </c>
+      <c r="G66" t="n">
+        <v>17272</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>61</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>FOCO FARMA</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>62</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>FOCO PILHAS</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>28</v>
+      </c>
+      <c r="G68" t="n">
+        <v>4811.68</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>62</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>FOCO SANDÁLIAS</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>62</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>FOCO HIGIENE</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>57</v>
+      </c>
+      <c r="G70" t="n">
+        <v>12739.52</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>62</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>FOCO ESPONJAS</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>62</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>FOCO CABELOS</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>70</v>
+      </c>
+      <c r="G72" t="n">
+        <v>16782.58</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>62</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>FOCO FARMA</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: pasta conta as vendas da equipe dela e evolução mostra dia e mês
A pasta passa a somar o que os vendedores dela venderam (letra no começo do
nome na 8081), de qualquer fornecedor; o total continua com tudo. Vendedor sem
pasta no nome cai na pasta do fornecedor, com aviso.

O gráfico de evolução agora mostra cada dia contra a meta do dia (barras) e o
mês acumulado contra o esperado (linha), com o % do mês na ponta.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015TKaSn4L8db77LPKSsZ5hm
</commit_message>
<xml_diff>
--- a/tools/exemplos/(BASE) - Metas Polybalas - KPI's e Produtos Focos.xlsx
+++ b/tools/exemplos/(BASE) - Metas Polybalas - KPI's e Produtos Focos.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,12 +467,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VENDEDOR 01</t>
+          <t>A-XX-01- VENDEDOR A1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>VENDEDOR 01</t>
+          <t>A-XX-01- VENDEDOR A1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -526,12 +526,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>VENDEDOR 01</t>
+          <t>A-XX-01- VENDEDOR A1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -557,12 +557,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VENDEDOR 01</t>
+          <t>A-XX-01- VENDEDOR A1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -585,12 +585,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>VENDEDOR 01</t>
+          <t>A-XX-01- VENDEDOR A1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -616,12 +616,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>VENDEDOR 01</t>
+          <t>A-XX-01- VENDEDOR A1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -644,12 +644,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>VENDEDOR 02</t>
+          <t>A-XX-02- VENDEDOR A2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -675,12 +675,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>VENDEDOR 02</t>
+          <t>A-XX-02- VENDEDOR A2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>VENDEDOR 02</t>
+          <t>A-XX-02- VENDEDOR A2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -734,12 +734,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>VENDEDOR 02</t>
+          <t>A-XX-02- VENDEDOR A2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -762,12 +762,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VENDEDOR 02</t>
+          <t>A-XX-02- VENDEDOR A2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>VENDEDOR 02</t>
+          <t>A-XX-02- VENDEDOR A2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>A-XX (SUPERVISOR A)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VENDEDOR 03</t>
+          <t>B-XX-01- VENDEDOR B1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -852,12 +852,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>VENDEDOR 03</t>
+          <t>B-XX-01- VENDEDOR B1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -880,12 +880,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>VENDEDOR 03</t>
+          <t>B-XX-01- VENDEDOR B1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -911,12 +911,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>VENDEDOR 03</t>
+          <t>B-XX-01- VENDEDOR B1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -939,12 +939,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>VENDEDOR 03</t>
+          <t>B-XX-01- VENDEDOR B1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -970,12 +970,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>VENDEDOR 03</t>
+          <t>B-XX-01- VENDEDOR B1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -998,12 +998,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>VENDEDOR 04</t>
+          <t>B-XX-02- VENDEDOR B2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1029,12 +1029,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>VENDEDOR 04</t>
+          <t>B-XX-02- VENDEDOR B2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>VENDEDOR 04</t>
+          <t>B-XX-02- VENDEDOR B2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1088,12 +1088,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>VENDEDOR 04</t>
+          <t>B-XX-02- VENDEDOR B2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1116,12 +1116,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>VENDEDOR 04</t>
+          <t>B-XX-02- VENDEDOR B2</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1147,12 +1147,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>VENDEDOR 04</t>
+          <t>B-XX-02- VENDEDOR B2</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>B-XX (SUPERVISOR B)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>VENDEDOR 05</t>
+          <t>C-XX-01- VENDEDOR C1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>VENDEDOR 05</t>
+          <t>C-XX-01- VENDEDOR C1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1234,12 +1234,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>VENDEDOR 05</t>
+          <t>C-XX-01- VENDEDOR C1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>VENDEDOR 05</t>
+          <t>C-XX-01- VENDEDOR C1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>VENDEDOR 05</t>
+          <t>C-XX-01- VENDEDOR C1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1324,12 +1324,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>VENDEDOR 05</t>
+          <t>C-XX-01- VENDEDOR C1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>VENDEDOR 06</t>
+          <t>C-XX-02- VENDEDOR C2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>VENDEDOR 06</t>
+          <t>C-XX-02- VENDEDOR C2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>VENDEDOR 06</t>
+          <t>C-XX-02- VENDEDOR C2</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1442,12 +1442,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>VENDEDOR 06</t>
+          <t>C-XX-02- VENDEDOR C2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1470,12 +1470,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>VENDEDOR 06</t>
+          <t>C-XX-02- VENDEDOR C2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>VENDEDOR 06</t>
+          <t>C-XX-02- VENDEDOR C2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>C-XX (SUPERVISOR C)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1529,12 +1529,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>VENDEDOR 07</t>
+          <t>D-XX-01- VENDEDOR D1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1560,12 +1560,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>VENDEDOR 07</t>
+          <t>D-XX-01- VENDEDOR D1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1588,12 +1588,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>VENDEDOR 07</t>
+          <t>D-XX-01- VENDEDOR D1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1619,12 +1619,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>VENDEDOR 07</t>
+          <t>D-XX-01- VENDEDOR D1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>VENDEDOR 07</t>
+          <t>D-XX-01- VENDEDOR D1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1678,12 +1678,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>VENDEDOR 07</t>
+          <t>D-XX-01- VENDEDOR D1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1706,12 +1706,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>VENDEDOR 08</t>
+          <t>D-XX-02- VENDEDOR D2</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1737,12 +1737,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>VENDEDOR 08</t>
+          <t>D-XX-02- VENDEDOR D2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>VENDEDOR 08</t>
+          <t>D-XX-02- VENDEDOR D2</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1796,12 +1796,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>VENDEDOR 08</t>
+          <t>D-XX-02- VENDEDOR D2</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1824,12 +1824,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>VENDEDOR 08</t>
+          <t>D-XX-02- VENDEDOR D2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VENDEDOR 08</t>
+          <t>D-XX-02- VENDEDOR D2</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>SUPERVISOR Z</t>
+          <t>D-XX (SUPERVISOR D)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1883,12 +1883,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VENDEDOR 09</t>
+          <t>E-XX-01- VENDEDOR E1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VENDEDOR 09</t>
+          <t>E-XX-01- VENDEDOR E1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1942,12 +1942,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>VENDEDOR 09</t>
+          <t>E-XX-01- VENDEDOR E1</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1973,12 +1973,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>VENDEDOR 09</t>
+          <t>E-XX-01- VENDEDOR E1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2001,12 +2001,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>VENDEDOR 09</t>
+          <t>E-XX-01- VENDEDOR E1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2032,12 +2032,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>VENDEDOR 09</t>
+          <t>E-XX-01- VENDEDOR E1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SUPERVISOR X</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2060,12 +2060,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>VENDEDOR 10</t>
+          <t>E-XX-02- VENDEDOR E2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2091,12 +2091,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VENDEDOR 10</t>
+          <t>E-XX-02- VENDEDOR E2</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2119,12 +2119,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>VENDEDOR 10</t>
+          <t>E-XX-02- VENDEDOR E2</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2150,12 +2150,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VENDEDOR 10</t>
+          <t>E-XX-02- VENDEDOR E2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2178,12 +2178,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>VENDEDOR 10</t>
+          <t>E-XX-02- VENDEDOR E2</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2209,12 +2209,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>VENDEDOR 10</t>
+          <t>E-XX-02- VENDEDOR E2</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SUPERVISOR Y</t>
+          <t>E-XX (SUPERVISOR E)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2233,16 +2233,16 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 61</t>
+          <t>F-XX-01- VENDEDOR F1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2264,16 +2264,16 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 61</t>
+          <t>F-XX-01- VENDEDOR F1</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2292,16 +2292,16 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 61</t>
+          <t>F-XX-01- VENDEDOR F1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2323,16 +2323,16 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 61</t>
+          <t>F-XX-01- VENDEDOR F1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2351,16 +2351,16 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 61</t>
+          <t>F-XX-01- VENDEDOR F1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2382,16 +2382,16 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 61</t>
+          <t>F-XX-01- VENDEDOR F1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2410,16 +2410,16 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 62</t>
+          <t>F-XX-02- VENDEDOR F2</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2441,16 +2441,16 @@
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 62</t>
+          <t>F-XX-02- VENDEDOR F2</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2469,16 +2469,16 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 62</t>
+          <t>F-XX-02- VENDEDOR F2</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2500,16 +2500,16 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 62</t>
+          <t>F-XX-02- VENDEDOR F2</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2528,16 +2528,16 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 62</t>
+          <t>F-XX-02- VENDEDOR F2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2559,16 +2559,16 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>P-TLV- VENDEDOR 62</t>
+          <t>F-XX-02- VENDEDOR F2</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+          <t>F-XX (SUPERVISOR F)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2583,6 +2583,714 @@
       </c>
       <c r="F73" t="n">
         <v>95</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>23</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>G-XX-01- VENDEDOR G1</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>FOCO PILHAS</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>31</v>
+      </c>
+      <c r="G74" t="n">
+        <v>3386.65</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>23</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>G-XX-01- VENDEDOR G1</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>FOCO SANDÁLIAS</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>23</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>G-XX-01- VENDEDOR G1</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>FOCO HIGIENE</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>48</v>
+      </c>
+      <c r="G76" t="n">
+        <v>9595.16</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>23</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>G-XX-01- VENDEDOR G1</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>FOCO ESPONJAS</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>23</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>G-XX-01- VENDEDOR G1</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>FOCO CABELOS</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>70</v>
+      </c>
+      <c r="G78" t="n">
+        <v>9002.57</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>23</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>G-XX-01- VENDEDOR G1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>FOCO FARMA</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>24</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>G-XX-02- VENDEDOR G2</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>FOCO PILHAS</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>26</v>
+      </c>
+      <c r="G80" t="n">
+        <v>3991.35</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>24</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>G-XX-02- VENDEDOR G2</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>FOCO SANDÁLIAS</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>24</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>G-XX-02- VENDEDOR G2</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>FOCO HIGIENE</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>52</v>
+      </c>
+      <c r="G82" t="n">
+        <v>11347.82</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>24</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>G-XX-02- VENDEDOR G2</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>FOCO ESPONJAS</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>24</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>G-XX-02- VENDEDOR G2</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>FOCO CABELOS</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>72</v>
+      </c>
+      <c r="G84" t="n">
+        <v>9061.57</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>24</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>G-XX-02- VENDEDOR G2</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>G-XX (SUPERVISOR G)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>FOCO FARMA</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>61</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>FOCO PILHAS</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>24</v>
+      </c>
+      <c r="G86" t="n">
+        <v>5183.21</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>61</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>FOCO SANDÁLIAS</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>61</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>FOCO HIGIENE</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>48</v>
+      </c>
+      <c r="G88" t="n">
+        <v>13666.22</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>61</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>FOCO ESPONJAS</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>61</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>FOCO CABELOS</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>77</v>
+      </c>
+      <c r="G90" t="n">
+        <v>10013.2</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>61</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 61</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>FOCO FARMA</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>62</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>FOCO PILHAS</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>24</v>
+      </c>
+      <c r="G92" t="n">
+        <v>6133.75</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>62</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>FOCO SANDÁLIAS</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>62</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>FOCO HIGIENE</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>60</v>
+      </c>
+      <c r="G94" t="n">
+        <v>9296.309999999999</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>62</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>FOCO ESPONJAS</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>VAREJO</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>62</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>FOCO CABELOS</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>84</v>
+      </c>
+      <c r="G96" t="n">
+        <v>18682.89</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>62</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>P-TLV- VENDEDOR 62</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>P-TELEVENDAS (SUPERVISOR T)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>FOCO FARMA</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>FARMA</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: pasta do vendedor pelo supervisor da 8081
O supervisor passa a ser a referência da pasta ("A-XX (...)", "G- FARMA (...)"
do Canal Farma, "P-TELEVENDAS (...)"); o nome do vendedor fica de reserva.
</commit_message>
<xml_diff>
--- a/tools/exemplos/(BASE) - Metas Polybalas - KPI's e Produtos Focos.xlsx
+++ b/tools/exemplos/(BASE) - Metas Polybalas - KPI's e Produtos Focos.xlsx
@@ -2596,7 +2596,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>G-XX (SUPERVISOR G)</t>
+          <t>G- FARMA (SUPERVISOR G)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">

</xml_diff>